<commit_message>
Update 퍼스널컬러 sheet: 22 businesses across 9 Seoul districts
</commit_message>
<xml_diff>
--- a/packages/명동_업체리스트.xlsx
+++ b/packages/명동_업체리스트.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="업체리스트_명동중심" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eSIM_여행자보험" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리_요약" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼스널컬러_서울전체" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="업체리스트_명동중심" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eSIM_여행자보험" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="카테고리_요약" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -105,7 +106,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -127,11 +128,25 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -164,6 +179,36 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -531,6 +576,996 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>거점</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>업체명</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>전화번호</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>인스타그램</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>주소</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>가까운 역</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>가격대</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>명동</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>컬러라이즈 명동본점</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>02-587-5205</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>@colorize_you</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>서울 중구 퇴계로 145, 세종호텔 별관 1층</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="inlineStr">
+        <is>
+          <t>명동역</t>
+        </is>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>₩45,000~(그룹)</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="inlineStr">
+        <is>
+          <t>1:1/그룹 선택. Klook 예약 가능. 외국어 대응. 09~22시</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>명동</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>컬러라이즈 명동2점</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>02-587-5205</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>@colorize_you</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>서울 중구 명동8가길 32, 6층</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>명동역</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>₩45,000~(그룹)</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>동일 브랜드 명동 2호점. 네이버 리뷰 5천건+ 4.9점</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>명동</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>코코리 명동점</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>02-587-9022</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>@cocory_personalcolor</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>서울 중구 명동 인근 (예약 시 안내)</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>명동역</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>₩80,000~</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>영·중·일 통역 가능. 네이버 예약. 색채학 기반 1:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>명동</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>컬러피윤</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>당근마켓 채널</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>당근마켓 채널</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>서울 중구 명동 (명동역 도보 5분)</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>명동역</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>별도 문의</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>9년차 MA 운영. 진단 후 립 시술 연계 가능</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>강남</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>컬러라이즈 강남점</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>02-587-5205</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>@colorize_you</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>서울 서초구 사임당로 173, 서전빌딩 4·9층</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>강남역</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>₩45,000~(그룹)</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>1:1/그룹 선택</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>강남</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>컬러플레이스</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>02-3443-5461</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>@colorplace_official</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>서울 강남구 봉은사로30길 54, 5층 (역삼동)</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>역삼역</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>₩100,000~(수석) / ₩350,000(대표)</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>프리미엄 1:1 전문. 인스타 팔로워 52K</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>강남</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>오콜로르 강남점</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>1800-6355</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>@colozart (colozart.com)</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>서울 강남구 논현로149길 52, 3층 (논현동)</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>학동역</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>₩130,000 (1인) / ₩190,000 (2인)</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>체형·골격진단 연계. Klook 등록. 영어 가능</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>압구정</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>오콜로르 신사점</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>1800-6355</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>@colozart (colozart.com)</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>서울 강남구 강남대로156길 20, 2층</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>신논현역</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>₩130,000 (1인)</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>퍼스널핏·체형컨설팅 연계</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>압구정</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>이미지호 가로수길점</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>imageho.co.kr 예약</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>@imageho_color_official</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>서울 강남구 압구정로10길 30-9, 4층</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>신사역</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>마이리얼트립 예약</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>외국어 가능. 진단 후 쇼핑 동반 서비스</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>홍대</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>컬러오브유</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>인스타 DM</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>@color_of_you_</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>서울 마포구 동교로 209, 용평빌딩 3층</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>홍대입구역 2번출구</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Klook/KKday 예약</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>영·중·일 통역 특화. 11~20시</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>홍대</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>코코리 홍대점</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>02-587-9022</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>@cocory.hongdae</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>서울 마포구 홍익로 11, 타입일레븐 3층</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>홍대입구역</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>₩80,000~</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>1:1. 네이버 예약 가능</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>홍대</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>컬러가산다</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>010-7287-9757</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>@colorgasanda_official</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>서울 마포구 동교로 192-1, 3층 (동교동)</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>홍대입구역</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>₩60,000(평일) / ₩65,000(주말)</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>2인 ₩100,000. 홈페이지 예약</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>홍대</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>담쁨</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>인스타 DM</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>@damppeum_</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>서울 마포구 홍대 인근 (DM 안내)</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>홍대입구역</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>₩80,000</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>드레이핑 전용. 측색기 미사용</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>합정</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>세컨뉴</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>인스타 DM</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>@seconew_color</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>서울 마포구 어울마당로 96, 5층</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>합정역</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>별도 문의</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>누적 3,000명+. 색채심리상담사 운영</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>신촌</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>위드컬러랑</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>인스타 DM</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>서울 용산구 백범로 8, 우정마샹스오피스텔 3층 339호</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>효창공원앞역</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>별도 문의</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>소형 프라이빗 스튜디오</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>성수</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>컬러츄</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>카카오채널</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>@color.chuu</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>서울 성동구 성수동 (성수역 도보 2분)</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>성수역</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>별도 문의</t>
+        </is>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>연 2,000명+. 200색 드레이핑. 대표 직접 진단</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>성수</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>코코리 성수점</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>02-587-9022</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>@cocory_seongsu</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>서울 성동구 성수 인근 (예약 시 안내)</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>성수역</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>₩80,000~</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>Klook 단독 페이지. 영어 가능</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>성수</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>컬러버랩</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>070-4949-7545</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>@colorloverlab_official</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>서울 성동구 성수이로 51, 서울숲한라시그마밸리 1동 13층 1302호</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>뚝섬역</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>₩25,000~</t>
+        </is>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>AI 앱 연동. 가성비 특화. 카카오채널 예약</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>성수</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>아름별컬러</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>0507-1328-8808</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>확인필요</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>서울 성동구 성수동1가 656-1158, 7층</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>성수역</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>별도 문의</t>
+        </is>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>16타입 진단. Waug 플랫폼 등록</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>용산</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>퍼스널컬러아카데미</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>02-6482-2890</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>별도 문의</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>서울 용산구 한강로2가 71</t>
+        </is>
+      </c>
+      <c r="F21" s="20" t="inlineStr">
+        <is>
+          <t>삼각지역</t>
+        </is>
+      </c>
+      <c r="G21" s="20" t="inlineStr">
+        <is>
+          <t>별도 문의</t>
+        </is>
+      </c>
+      <c r="H21" s="20" t="inlineStr">
+        <is>
+          <t>매일 10~20시. 자격증 교육 병행</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>잠실</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>컬러마인</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>인스타 DM</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>@color.mine</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="inlineStr">
+        <is>
+          <t>서울 송파구 잠실 인근 (예약 시 안내)</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>잠실역</t>
+        </is>
+      </c>
+      <c r="G22" s="21" t="inlineStr">
+        <is>
+          <t>별도 문의</t>
+        </is>
+      </c>
+      <c r="H22" s="21" t="inlineStr">
+        <is>
+          <t>골격진단·웨딩 연계. 11~18시</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>잠실</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>컬러정</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>솜씨당 예약</t>
+        </is>
+      </c>
+      <c r="D23" s="21" t="inlineStr">
+        <is>
+          <t>솜씨당 채널</t>
+        </is>
+      </c>
+      <c r="E23" s="21" t="inlineStr">
+        <is>
+          <t>서울 송파구 잠실동 27-8</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr">
+        <is>
+          <t>잠실새내역</t>
+        </is>
+      </c>
+      <c r="G23" s="21" t="inlineStr">
+        <is>
+          <t>별도 문의</t>
+        </is>
+      </c>
+      <c r="H23" s="21" t="inlineStr">
+        <is>
+          <t>21타입 188색 천. 총 70분</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3011,7 +4046,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3441,7 +4476,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>